<commit_message>
wip(G1): A01 constraints come only from its authorization record; Gain Access recorded in the Session Planning Model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/back/data/session-planning/session-planning-model.rc1.xlsx
+++ b/back/data/session-planning/session-planning-model.rc1.xlsx
@@ -6418,11 +6418,15 @@
           <t>A01</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>GP-005</t>
+        </is>
+      </c>
       <c r="C2" s="4" t="n"/>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Intentional runtime gap (Cycle 8 §5) — no placeholder mapping. Runtime realization opportunity, not a knowledge deficiency.</t>
+          <t>Approved 2026-10-15 (Christian, A01 decision 1) — Primary Representative Game Problem Translation: Gain Access, based on the approved Goalkeeper Build-Out context (RPC-001) and its scoring condition. No secondary (Cycle 8 §4 deferral retained). Replaces the Cycle 8 §5 intentional runtime gap. Does not by itself authorize candidate constraints derived from vocabulary coverage.</t>
         </is>
       </c>
     </row>

</xml_diff>